<commit_message>
Refonte portfolio: ajout Pizzeria + Capgemini, badges, banner Open to Work, fixs liens
- Ajout projet Pizzeria Bella Italia avec lien live (Stage Mambo 2e annee)
- Ajout projet Capgemini MQTT POC (Stage 1ere annee)
- Banner Open to Work alternance DevOps/IA Septembre 2026
- Skill bars % remplaces par skill-badges (plus pro, plus de pourcentages subjectifs)
- Footer dynamique: annee auto + lien GitHub + LinkedIn
- Fix lien GLPI casse (GLPI/ vers glpi/ - sensible a la casse sur Linux)
- Fix lien LinkedIn casse (#) avec vraie URL
- Ajout contact GitHub
- Mise a jour stats: 8 projets, 3 stages, 12+ technos
- Dates projets BTS: 2024-2025 vers 2025-2026 (2e annee)
- Synthese: ajout ligne Pizzeria Bella Italia, retrait Polaris (etait BTS SNIR)
- Tableau Excel synthese mis a jour (docs/tableau_synthese_2025.xlsx)
</commit_message>
<xml_diff>
--- a/docs/tableau_synthese_2025.xlsx
+++ b/docs/tableau_synthese_2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29728"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/okacha/Downloads/Promo_300_26/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dieng\Downloads\cv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_F9CA3684FE8986572AEDD281E351102199C0AD04" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E5BCA58D-9277-45E9-AD96-024C73C49472}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="820" yWindow="500" windowWidth="19740" windowHeight="12460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tableau de synthèse Épreuve E4" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="42">
   <si>
     <t>BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
   </si>
@@ -57,15 +57,6 @@
     <t xml:space="preserve">Tableau de synthèse des réalisations professionnelles </t>
   </si>
   <si>
-    <t>NOM et prénom :</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N° candidat : </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Centre de formation : </t>
-  </si>
-  <si>
     <t>Option :</t>
   </si>
   <si>
@@ -73,9 +64,6 @@
   </si>
   <si>
     <t>X SLAM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Adresse URL Portfolio : </t>
   </si>
   <si>
     <t>Compétences mises en œuvre
@@ -142,31 +130,67 @@
 </t>
   </si>
   <si>
-    <t>Installation et configuration d'un serveur Linux virtualisé avec la gestion des incidents GLPI</t>
-  </si>
-  <si>
-    <t>Conception et développement du site internet E-Ensiegnement avec le CMS WordPresse</t>
-  </si>
-  <si>
-    <t>Développement du jeu ….. en Langage C avec Git_GitHub en mode projet</t>
-  </si>
-  <si>
-    <t>Formation Certification en …</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Elaboration d'une veille technologique sur ….</t>
-  </si>
-  <si>
-    <t>Développement du site marchant …. Avec le CMS Shopify en mode Projet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Conception et développement du site internet Cabinet médical </t>
-  </si>
-  <si>
     <t>Réalisations en milieu professionnel en cours de première année</t>
   </si>
   <si>
     <t>Réalisations en milieu professionnel en cours de seconde année</t>
+  </si>
+  <si>
+    <t>NOM et prénom : DIENG Mouhammad El Bachir</t>
+  </si>
+  <si>
+    <t>N° candidat : 02544742622</t>
+  </si>
+  <si>
+    <t>Centre de formation : IRIS PARIS</t>
+  </si>
+  <si>
+    <t>Adresse URL Portfolio : https://melbachirdieng.github.io/</t>
+  </si>
+  <si>
+    <t>Installation et configuration d'un serveur Linux virtualisé avec gestion des incidents GLPI</t>
+  </si>
+  <si>
+    <t>Sep-25</t>
+  </si>
+  <si>
+    <t>Conception et développement du site internet E-Enseignement avec le CMS WordPress</t>
+  </si>
+  <si>
+    <t>Développement du jeu Snake en Langage C avec Git/GitHub en mode projet</t>
+  </si>
+  <si>
+    <t>Oct-25</t>
+  </si>
+  <si>
+    <t>Formations Certifications en Python et WordPress</t>
+  </si>
+  <si>
+    <t>Jan-25 à avril-26</t>
+  </si>
+  <si>
+    <t>Élaboration d'une veille technologique sur le DevOps, l'IA générative et la cybersécurité</t>
+  </si>
+  <si>
+    <t>Développement du site marchand JuiceLab avec le CMS Shopify en mode projet</t>
+  </si>
+  <si>
+    <t>Conception et développement du site internet Auto-école en HTML/CSS et PHP/MySQL</t>
+  </si>
+  <si>
+    <t>Nov-25</t>
+  </si>
+  <si>
+    <t>Stage Capgemini Technology Services : développement Python (paho-mqtt) et déploiement broker Apache ActiveMQ pour simulation MES (Manufacturing Execution System)</t>
+  </si>
+  <si>
+    <t>Du 21/07/2025 au 29/08/2025 (6 semaines)</t>
+  </si>
+  <si>
+    <t>Stage Mambo Inchaud Conception de Site Web : conception et développement d'un site vitrine de pizzeria (Pizzeria Bella Italia) en HTML/CSS, JS, PHP 8, MySQL/PDO avec back-office admin sécurisé</t>
+  </si>
+  <si>
+    <t>Du 17/11/2025 au 19/12/2025 (5 semaines)</t>
   </si>
 </sst>
 </file>
@@ -176,7 +200,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-1]_-;\-* #,##0.00\ [$€-1]_-;_-* &quot;-&quot;??\ [$€-1]_-"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -266,13 +290,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0"/>
+        <fgColor rgb="FF70CF47"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -622,7 +646,7 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -630,18 +654,12 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -657,104 +675,125 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="17" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="17" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1067,134 +1106,134 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AQ66"/>
-  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="12.95"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.88671875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="70.42578125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="22.28515625" style="1" customWidth="1"/>
-    <col min="3" max="8" width="18.7109375" style="1" customWidth="1"/>
-    <col min="9" max="43" width="11.42578125" customWidth="1"/>
-    <col min="44" max="16384" width="10.85546875" style="1"/>
+    <col min="1" max="1" width="70.44140625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="22.33203125" style="1" customWidth="1"/>
+    <col min="3" max="8" width="18.6640625" style="1" customWidth="1"/>
+    <col min="9" max="43" width="11.44140625" customWidth="1"/>
+    <col min="44" max="16384" width="10.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" ht="39.950000000000003" customHeight="1">
-      <c r="A1" s="23" t="s">
+    <row r="1" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23" t="s">
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="23"/>
+      <c r="H1" s="15"/>
     </row>
-    <row r="2" spans="1:43" ht="41.1" customHeight="1">
-      <c r="A2" s="23" t="s">
+    <row r="2" spans="1:43" ht="41.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="23"/>
-      <c r="H2" s="23"/>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
     </row>
-    <row r="3" spans="1:43" ht="39.950000000000003" customHeight="1">
-      <c r="A3" s="24" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="25"/>
-      <c r="C3" s="25"/>
-      <c r="D3" s="25"/>
-      <c r="E3" s="26"/>
-      <c r="F3" s="30" t="s">
-        <v>4</v>
-      </c>
-      <c r="G3" s="31"/>
-      <c r="H3" s="32"/>
+    <row r="3" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" s="17"/>
+      <c r="C3" s="17"/>
+      <c r="D3" s="17"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="G3" s="23"/>
+      <c r="H3" s="24"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
-    <row r="4" spans="1:43" ht="39.950000000000003" customHeight="1">
-      <c r="A4" s="27" t="s">
+    <row r="4" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="H4" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="28"/>
-      <c r="C4" s="28"/>
-      <c r="D4" s="28"/>
-      <c r="E4" s="29"/>
-      <c r="F4" s="7" t="s">
+    </row>
+    <row r="5" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="34" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="35"/>
+      <c r="C5" s="35"/>
+      <c r="D5" s="35"/>
+      <c r="E5" s="35"/>
+      <c r="F5" s="35"/>
+      <c r="G5" s="35"/>
+      <c r="H5" s="36"/>
+    </row>
+    <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="G4" s="8" t="s">
+      <c r="B6" s="32" t="s">
         <v>7</v>
       </c>
-      <c r="H4" s="9" t="s">
+      <c r="C6" s="8" t="s">
         <v>8</v>
       </c>
+      <c r="D6" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H6" s="9" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row r="5" spans="1:43" ht="39.950000000000003" customHeight="1">
-      <c r="A5" s="42" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" s="43"/>
-      <c r="C5" s="43"/>
-      <c r="D5" s="43"/>
-      <c r="E5" s="43"/>
-      <c r="F5" s="43"/>
-      <c r="G5" s="43"/>
-      <c r="H5" s="44"/>
-    </row>
-    <row r="6" spans="1:43" ht="90" customHeight="1">
-      <c r="A6" s="33" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="40" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="E6" s="10" t="s">
+    <row r="7" spans="1:43" s="2" customFormat="1" ht="324.89999999999998" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="25"/>
+      <c r="B7" s="33"/>
+      <c r="C7" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="F6" s="10" t="s">
+      <c r="D7" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="G6" s="10" t="s">
+      <c r="E7" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="H6" s="11" t="s">
+      <c r="F7" s="11" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="7" spans="1:43" s="2" customFormat="1" ht="324.95" customHeight="1" thickBot="1">
-      <c r="A7" s="33"/>
-      <c r="B7" s="41"/>
-      <c r="C7" s="19" t="s">
+      <c r="G7" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="19" t="s">
+      <c r="H7" s="12" t="s">
         <v>19</v>
-      </c>
-      <c r="E7" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="F7" s="19" t="s">
-        <v>21</v>
-      </c>
-      <c r="G7" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="H7" s="20" t="s">
-        <v>23</v>
       </c>
       <c r="I7"/>
       <c r="J7"/>
@@ -1232,17 +1271,17 @@
       <c r="AP7"/>
       <c r="AQ7"/>
     </row>
-    <row r="8" spans="1:43" s="2" customFormat="1" ht="18">
-      <c r="A8" s="34" t="s">
-        <v>24</v>
-      </c>
-      <c r="B8" s="35"/>
-      <c r="C8" s="35"/>
-      <c r="D8" s="35"/>
-      <c r="E8" s="35"/>
-      <c r="F8" s="35"/>
-      <c r="G8" s="35"/>
-      <c r="H8" s="36"/>
+    <row r="8" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
+      <c r="A8" s="26" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="27"/>
+      <c r="C8" s="27"/>
+      <c r="D8" s="27"/>
+      <c r="E8" s="27"/>
+      <c r="F8" s="27"/>
+      <c r="G8" s="27"/>
+      <c r="H8" s="28"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1279,19 +1318,19 @@
       <c r="AP8"/>
       <c r="AQ8"/>
     </row>
-    <row r="9" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
-      <c r="A9" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="B9" s="15">
-        <v>45901</v>
-      </c>
-      <c r="C9" s="12"/>
-      <c r="D9" s="13"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="13"/>
-      <c r="G9" s="13"/>
-      <c r="H9" s="6"/>
+    <row r="9" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="40" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" s="41" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" s="42"/>
+      <c r="D9" s="43"/>
+      <c r="E9" s="38"/>
+      <c r="F9" s="43"/>
+      <c r="G9" s="43"/>
+      <c r="H9" s="39"/>
       <c r="I9"/>
       <c r="J9"/>
       <c r="K9"/>
@@ -1328,19 +1367,19 @@
       <c r="AP9"/>
       <c r="AQ9"/>
     </row>
-    <row r="10" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
-      <c r="A10" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="B10" s="15">
-        <v>45901</v>
-      </c>
-      <c r="C10" s="12"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="13"/>
-      <c r="F10" s="13"/>
-      <c r="G10" s="13"/>
-      <c r="H10" s="6"/>
+    <row r="10" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="40" t="s">
+        <v>29</v>
+      </c>
+      <c r="B10" s="41" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" s="37"/>
+      <c r="D10" s="38"/>
+      <c r="E10" s="43"/>
+      <c r="F10" s="43"/>
+      <c r="G10" s="43"/>
+      <c r="H10" s="39"/>
       <c r="I10"/>
       <c r="J10"/>
       <c r="K10"/>
@@ -1377,19 +1416,19 @@
       <c r="AP10"/>
       <c r="AQ10"/>
     </row>
-    <row r="11" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
-      <c r="A11" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="B11" s="15">
-        <v>45931</v>
-      </c>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="13"/>
-      <c r="G11" s="13"/>
-      <c r="H11" s="6"/>
+    <row r="11" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="40" t="s">
+        <v>30</v>
+      </c>
+      <c r="B11" s="41" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" s="38"/>
+      <c r="D11" s="38"/>
+      <c r="E11" s="38"/>
+      <c r="F11" s="43"/>
+      <c r="G11" s="43"/>
+      <c r="H11" s="39"/>
       <c r="I11"/>
       <c r="J11"/>
       <c r="K11"/>
@@ -1426,17 +1465,19 @@
       <c r="AP11"/>
       <c r="AQ11"/>
     </row>
-    <row r="12" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
-      <c r="A12" s="14" t="s">
-        <v>28</v>
-      </c>
-      <c r="B12" s="15"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
-      <c r="H12" s="16"/>
+    <row r="12" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="40" t="s">
+        <v>32</v>
+      </c>
+      <c r="B12" s="41" t="s">
+        <v>33</v>
+      </c>
+      <c r="C12" s="38"/>
+      <c r="D12" s="38"/>
+      <c r="E12" s="38"/>
+      <c r="F12" s="38"/>
+      <c r="G12" s="38"/>
+      <c r="H12" s="44"/>
       <c r="I12"/>
       <c r="J12"/>
       <c r="K12"/>
@@ -1473,19 +1514,19 @@
       <c r="AP12"/>
       <c r="AQ12"/>
     </row>
-    <row r="13" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
-      <c r="A13" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="B13" s="15">
-        <v>45352</v>
-      </c>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5"/>
-      <c r="H13" s="16"/>
+    <row r="13" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="40" t="s">
+        <v>34</v>
+      </c>
+      <c r="B13" s="41" t="s">
+        <v>31</v>
+      </c>
+      <c r="C13" s="38"/>
+      <c r="D13" s="38"/>
+      <c r="E13" s="38"/>
+      <c r="F13" s="38"/>
+      <c r="G13" s="38"/>
+      <c r="H13" s="44"/>
       <c r="I13"/>
       <c r="J13"/>
       <c r="K13"/>
@@ -1522,19 +1563,19 @@
       <c r="AP13"/>
       <c r="AQ13"/>
     </row>
-    <row r="14" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
-      <c r="A14" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B14" s="18">
-        <v>45597</v>
-      </c>
-      <c r="C14" s="5"/>
-      <c r="D14" s="13"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="13"/>
-      <c r="G14" s="13"/>
-      <c r="H14" s="6"/>
+    <row r="14" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="45" t="s">
+        <v>35</v>
+      </c>
+      <c r="B14" s="46" t="s">
+        <v>31</v>
+      </c>
+      <c r="C14" s="38"/>
+      <c r="D14" s="43"/>
+      <c r="E14" s="43"/>
+      <c r="F14" s="43"/>
+      <c r="G14" s="43"/>
+      <c r="H14" s="39"/>
       <c r="I14"/>
       <c r="J14"/>
       <c r="K14"/>
@@ -1571,19 +1612,19 @@
       <c r="AP14"/>
       <c r="AQ14"/>
     </row>
-    <row r="15" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
-      <c r="A15" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B15" s="18">
-        <v>45992</v>
-      </c>
-      <c r="C15" s="5"/>
-      <c r="D15" s="13"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="13"/>
-      <c r="G15" s="13"/>
-      <c r="H15" s="6"/>
+    <row r="15" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="45" t="s">
+        <v>36</v>
+      </c>
+      <c r="B15" s="46" t="s">
+        <v>37</v>
+      </c>
+      <c r="C15" s="38"/>
+      <c r="D15" s="38"/>
+      <c r="E15" s="43"/>
+      <c r="F15" s="43"/>
+      <c r="G15" s="43"/>
+      <c r="H15" s="39"/>
       <c r="I15"/>
       <c r="J15"/>
       <c r="K15"/>
@@ -1620,17 +1661,17 @@
       <c r="AP15"/>
       <c r="AQ15"/>
     </row>
-    <row r="16" spans="1:43" s="2" customFormat="1" ht="18">
-      <c r="A16" s="37" t="s">
-        <v>32</v>
-      </c>
-      <c r="B16" s="38"/>
-      <c r="C16" s="38"/>
-      <c r="D16" s="38"/>
-      <c r="E16" s="38"/>
-      <c r="F16" s="38"/>
-      <c r="G16" s="38"/>
-      <c r="H16" s="39"/>
+    <row r="16" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
+      <c r="A16" s="29" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16" s="30"/>
+      <c r="C16" s="30"/>
+      <c r="D16" s="30"/>
+      <c r="E16" s="30"/>
+      <c r="F16" s="30"/>
+      <c r="G16" s="30"/>
+      <c r="H16" s="31"/>
       <c r="I16"/>
       <c r="J16"/>
       <c r="K16"/>
@@ -1667,15 +1708,19 @@
       <c r="AP16"/>
       <c r="AQ16"/>
     </row>
-    <row r="17" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
-      <c r="A17" s="4"/>
-      <c r="B17" s="17"/>
-      <c r="C17" s="17"/>
-      <c r="D17" s="5"/>
-      <c r="E17" s="17"/>
-      <c r="F17" s="5"/>
-      <c r="G17" s="17"/>
-      <c r="H17" s="6"/>
+    <row r="17" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="45" t="s">
+        <v>38</v>
+      </c>
+      <c r="B17" s="46" t="s">
+        <v>39</v>
+      </c>
+      <c r="C17" s="48"/>
+      <c r="D17" s="38"/>
+      <c r="E17" s="47"/>
+      <c r="F17" s="43"/>
+      <c r="G17" s="48"/>
+      <c r="H17" s="44"/>
       <c r="I17"/>
       <c r="J17"/>
       <c r="K17"/>
@@ -1712,15 +1757,15 @@
       <c r="AP17"/>
       <c r="AQ17"/>
     </row>
-    <row r="18" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
-      <c r="A18" s="4"/>
-      <c r="B18" s="17"/>
-      <c r="C18" s="17"/>
-      <c r="D18" s="21"/>
-      <c r="E18" s="17"/>
-      <c r="F18" s="5"/>
-      <c r="G18" s="17"/>
-      <c r="H18" s="22"/>
+    <row r="18" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="3"/>
+      <c r="B18" s="10"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="4"/>
+      <c r="G18" s="10"/>
+      <c r="H18" s="14"/>
       <c r="I18"/>
       <c r="J18"/>
       <c r="K18"/>
@@ -1757,17 +1802,17 @@
       <c r="AP18"/>
       <c r="AQ18"/>
     </row>
-    <row r="19" spans="1:43" s="2" customFormat="1" ht="18">
-      <c r="A19" s="37" t="s">
-        <v>33</v>
-      </c>
-      <c r="B19" s="38"/>
-      <c r="C19" s="38"/>
-      <c r="D19" s="38"/>
-      <c r="E19" s="38"/>
-      <c r="F19" s="38"/>
-      <c r="G19" s="38"/>
-      <c r="H19" s="39"/>
+    <row r="19" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
+      <c r="A19" s="29" t="s">
+        <v>22</v>
+      </c>
+      <c r="B19" s="30"/>
+      <c r="C19" s="30"/>
+      <c r="D19" s="30"/>
+      <c r="E19" s="30"/>
+      <c r="F19" s="30"/>
+      <c r="G19" s="30"/>
+      <c r="H19" s="31"/>
       <c r="I19"/>
       <c r="J19"/>
       <c r="K19"/>
@@ -1804,15 +1849,19 @@
       <c r="AP19"/>
       <c r="AQ19"/>
     </row>
-    <row r="20" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
-      <c r="A20" s="4"/>
-      <c r="B20" s="3"/>
-      <c r="C20" s="5"/>
-      <c r="D20" s="17"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
-      <c r="G20" s="5"/>
-      <c r="H20" s="6"/>
+    <row r="20" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="45" t="s">
+        <v>40</v>
+      </c>
+      <c r="B20" s="49" t="s">
+        <v>41</v>
+      </c>
+      <c r="C20" s="38"/>
+      <c r="D20" s="47"/>
+      <c r="E20" s="43"/>
+      <c r="F20" s="43"/>
+      <c r="G20" s="43"/>
+      <c r="H20" s="39"/>
       <c r="I20"/>
       <c r="J20"/>
       <c r="K20"/>
@@ -1849,52 +1898,52 @@
       <c r="AP20"/>
       <c r="AQ20"/>
     </row>
-    <row r="21" spans="1:43" customFormat="1"/>
-    <row r="22" spans="1:43" customFormat="1"/>
-    <row r="23" spans="1:43" customFormat="1"/>
-    <row r="24" spans="1:43" customFormat="1"/>
-    <row r="25" spans="1:43" customFormat="1"/>
-    <row r="26" spans="1:43" customFormat="1"/>
-    <row r="27" spans="1:43" customFormat="1"/>
-    <row r="28" spans="1:43" customFormat="1"/>
-    <row r="29" spans="1:43" customFormat="1"/>
-    <row r="30" spans="1:43" customFormat="1"/>
-    <row r="31" spans="1:43" customFormat="1"/>
-    <row r="32" spans="1:43" customFormat="1"/>
-    <row r="33" customFormat="1"/>
-    <row r="34" customFormat="1"/>
-    <row r="35" customFormat="1"/>
-    <row r="36" customFormat="1"/>
-    <row r="37" customFormat="1"/>
-    <row r="38" customFormat="1"/>
-    <row r="39" customFormat="1"/>
-    <row r="40" customFormat="1"/>
-    <row r="41" customFormat="1"/>
-    <row r="42" customFormat="1"/>
-    <row r="43" customFormat="1"/>
-    <row r="44" customFormat="1"/>
-    <row r="45" customFormat="1"/>
-    <row r="46" customFormat="1"/>
-    <row r="47" customFormat="1"/>
-    <row r="48" customFormat="1"/>
-    <row r="49" customFormat="1"/>
-    <row r="50" customFormat="1"/>
-    <row r="51" customFormat="1"/>
-    <row r="52" customFormat="1"/>
-    <row r="53" customFormat="1"/>
-    <row r="54" customFormat="1"/>
-    <row r="55" customFormat="1"/>
-    <row r="56" customFormat="1"/>
-    <row r="57" customFormat="1"/>
-    <row r="58" customFormat="1"/>
-    <row r="59" customFormat="1"/>
-    <row r="60" customFormat="1"/>
-    <row r="61" customFormat="1"/>
-    <row r="62" customFormat="1"/>
-    <row r="63" customFormat="1"/>
-    <row r="64" customFormat="1"/>
-    <row r="65" customFormat="1"/>
-    <row r="66" customFormat="1"/>
+    <row r="21" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="22" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="23" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="24" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="25" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="27" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="28" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="29" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="30" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="31" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="32" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="33" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="34" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="35" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="36" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="37" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="38" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="39" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="40" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="41" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="42" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="44" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="45" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="46" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="47" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="48" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="49" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="50" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="51" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="52" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="53" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="54" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="55" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="56" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="57" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="58" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="59" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="60" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="61" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="62" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="63" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="64" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="65" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="66" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="12">
     <mergeCell ref="A6:A7"/>
@@ -1921,7 +1970,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.95"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2137,13 +2186,39 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{115E9D4D-BBFA-4016-A3EB-D1328016C37C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{115E9D4D-BBFA-4016-A3EB-D1328016C37C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="191d0fcf-6d89-4c90-807a-10f37b8d7a4c"/>
+    <ds:schemaRef ds:uri="9a7dc87b-2be1-4fee-871a-355a79ca984c"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B4B2C3C2-98C5-40C9-936C-A0749252C73F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B4B2C3C2-98C5-40C9-936C-A0749252C73F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="191d0fcf-6d89-4c90-807a-10f37b8d7a4c"/>
+    <ds:schemaRef ds:uri="9a7dc87b-2be1-4fee-871a-355a79ca984c"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{12891FC5-B985-42D8-BB15-5428EFF482F5}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{12891FC5-B985-42D8-BB15-5428EFF482F5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Veille IA basket + corrections dates synthese
- Section Veille: refocus sur l'IA dans le basketball (NBA/EuroLeague) avec sources et flux RSS (Sloan, NBA, Cleaning the Glass, Thinking Basketball, etc.)
- Synthese: dates corrigees pour matcher le xlsx officiel (Sep/Oct/Nov 2025)
- Cartes projets: dates precises au mois pres
- Ajout ligne Veille dans le tableau synthese
- Renommage Shopify -> JuiceLab (Shopify) pour matcher xlsx
- About: ajout du 3e stage (Mambo Inchaud) et orientation DevOps/IA
- Regen xlsx synthese avec nouveau sujet de veille

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tableau_synthese_2025.xlsx
+++ b/docs/tableau_synthese_2025.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dieng\Downloads\cv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E5BCA58D-9277-45E9-AD96-024C73C49472}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E2FC7729-CC67-4EEE-8B41-F11D2AB6047B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5748" yWindow="948" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tableau de synthèse Épreuve E4" sheetId="1" r:id="rId1"/>
@@ -169,7 +169,7 @@
     <t>Jan-25 à avril-26</t>
   </si>
   <si>
-    <t>Élaboration d'une veille technologique sur le DevOps, l'IA générative et la cybersécurité</t>
+    <t>Élaboration d'une veille technologique sur l'application de l'intelligence artificielle dans le basketball (NBA / EuroLeague)</t>
   </si>
   <si>
     <t>Développement du site marchand JuiceLab avec le CMS Shopify en mode projet</t>

</xml_diff>